<commit_message>
add correct file to pre-week 2
</commit_message>
<xml_diff>
--- a/pre-week-02/Homework2.xlsx
+++ b/pre-week-02/Homework2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alondramartinez\Documents\DataAnalytics\pre-week-02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C362584B-9D46-4BD7-A72E-0839F08FF959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{229015E9-42F8-491A-A6C5-11FD59D1C21C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E5364FFE-2114-481A-8F53-4D3C0F23314E}"/>
+    <workbookView xWindow="0" yWindow="408" windowWidth="14196" windowHeight="11976" xr2:uid="{E5364FFE-2114-481A-8F53-4D3C0F23314E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet_1" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
update new file to pre-week02
</commit_message>
<xml_diff>
--- a/pre-week-02/Homework2.xlsx
+++ b/pre-week-02/Homework2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alondramartinez\Documents\DataAnalytics\pre-week-02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E16F68D1-E9A3-4D7A-9FE8-E10E0900DFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{81CA4706-C6BA-4522-AE4F-A5F1E6888C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="408" windowWidth="14196" windowHeight="11976" xr2:uid="{E5364FFE-2114-481A-8F53-4D3C0F23314E}"/>
+    <workbookView xWindow="0" yWindow="408" windowWidth="14196" windowHeight="11976" activeTab="2" xr2:uid="{E5364FFE-2114-481A-8F53-4D3C0F23314E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet_1" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
fix homework2 file name and location
</commit_message>
<xml_diff>
--- a/pre-week-02/Homework2.xlsx
+++ b/pre-week-02/Homework2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alondramartinez\Documents\DataAnalytics\pre-week-02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{81CA4706-C6BA-4522-AE4F-A5F1E6888C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{49F21F44-2DB0-419A-B940-F72B011D0291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="408" windowWidth="14196" windowHeight="11976" activeTab="2" xr2:uid="{E5364FFE-2114-481A-8F53-4D3C0F23314E}"/>
+    <workbookView xWindow="4248" yWindow="1020" windowWidth="14196" windowHeight="11976" xr2:uid="{E5364FFE-2114-481A-8F53-4D3C0F23314E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet_1" sheetId="2" r:id="rId1"/>

</xml_diff>